<commit_message>
New file with the modified csv
</commit_message>
<xml_diff>
--- a/forPython.xlsx
+++ b/forPython.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Depalma-Lab/Alexia/3.Experiments/20251028-Thawing_Dcp_test/ThawingDCPs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C93B386A-0006-0049-9256-6AEE1FA5CC5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{062CC22B-D2DD-0340-92AF-32B232FD0B3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17040" activeTab="3" xr2:uid="{04F21ADD-521C-3D43-8BD2-2F70976D6201}"/>
   </bookViews>
@@ -247,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -267,6 +267,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7865,43 +7866,43 @@
       <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
-        <v>0</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0</v>
-      </c>
-      <c r="G3" s="2">
-        <v>0</v>
-      </c>
-      <c r="H3" s="2">
-        <v>0</v>
-      </c>
-      <c r="I3" s="2">
-        <v>0</v>
-      </c>
-      <c r="J3" s="2">
-        <v>0</v>
-      </c>
-      <c r="K3" s="2">
-        <v>0</v>
-      </c>
-      <c r="L3" s="2">
-        <v>0</v>
-      </c>
-      <c r="M3" s="3">
+      <c r="D3" s="15">
+        <v>0</v>
+      </c>
+      <c r="E3" s="15">
+        <v>0</v>
+      </c>
+      <c r="F3" s="15">
+        <v>0</v>
+      </c>
+      <c r="G3" s="15">
+        <v>0</v>
+      </c>
+      <c r="H3" s="15">
+        <v>0</v>
+      </c>
+      <c r="I3" s="15">
+        <v>0</v>
+      </c>
+      <c r="J3" s="15">
+        <v>0</v>
+      </c>
+      <c r="K3" s="15">
+        <v>0</v>
+      </c>
+      <c r="L3" s="15">
+        <v>0</v>
+      </c>
+      <c r="M3" s="15">
         <v>0.99399999999999999</v>
       </c>
-      <c r="N3" s="2">
-        <v>0</v>
-      </c>
-      <c r="O3" s="2">
-        <v>0</v>
-      </c>
-      <c r="P3" s="2">
+      <c r="N3" s="15">
+        <v>0</v>
+      </c>
+      <c r="O3" s="15">
+        <v>0</v>
+      </c>
+      <c r="P3" s="15">
         <v>0</v>
       </c>
     </row>
@@ -7912,43 +7913,43 @@
       <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="15">
         <v>9.9000000000000008E-3</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="15">
         <v>1.8E-3</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="15">
         <v>2.12E-2</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="15">
         <v>5.28E-2</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="15">
         <v>8.8000000000000003E-4</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="15">
         <v>1.95E-2</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="15">
         <v>2.2000000000000001E-4</v>
       </c>
-      <c r="K4" s="3">
+      <c r="K4" s="15">
         <v>8.4099999999999994E-2</v>
       </c>
-      <c r="L4" s="3">
+      <c r="L4" s="15">
         <v>6.6E-4</v>
       </c>
-      <c r="M4" s="3">
+      <c r="M4" s="15">
         <v>9.06E-2</v>
       </c>
-      <c r="N4" s="3">
+      <c r="N4" s="15">
         <v>0.21</v>
       </c>
-      <c r="O4" s="3">
+      <c r="O4" s="15">
         <v>7.2300000000000003E-2</v>
       </c>
-      <c r="P4" s="3">
+      <c r="P4" s="15">
         <v>0.157</v>
       </c>
     </row>
@@ -7959,43 +7960,43 @@
       <c r="C5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="15">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="E5" s="2">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2">
-        <v>0</v>
-      </c>
-      <c r="G5" s="2">
-        <v>0</v>
-      </c>
-      <c r="H5" s="2">
-        <v>0</v>
-      </c>
-      <c r="I5" s="4">
+      <c r="E5" s="15">
+        <v>0</v>
+      </c>
+      <c r="F5" s="15">
+        <v>0</v>
+      </c>
+      <c r="G5" s="15">
+        <v>0</v>
+      </c>
+      <c r="H5" s="15">
+        <v>0</v>
+      </c>
+      <c r="I5" s="15">
         <v>9.98E-5</v>
       </c>
-      <c r="J5" s="2">
-        <v>0</v>
-      </c>
-      <c r="K5" s="3">
+      <c r="J5" s="15">
+        <v>0</v>
+      </c>
+      <c r="K5" s="15">
         <v>2.5000000000000001E-4</v>
       </c>
-      <c r="L5" s="3">
+      <c r="L5" s="15">
         <v>4.7000000000000002E-3</v>
       </c>
-      <c r="M5" s="3">
+      <c r="M5" s="15">
         <v>0.66500000000000004</v>
       </c>
-      <c r="N5" s="3">
+      <c r="N5" s="15">
         <v>0.30299999999999999</v>
       </c>
-      <c r="O5" s="3">
+      <c r="O5" s="15">
         <v>5.5000000000000003E-4</v>
       </c>
-      <c r="P5" s="3">
+      <c r="P5" s="15">
         <v>1.6000000000000001E-3</v>
       </c>
     </row>
@@ -8006,43 +8007,43 @@
       <c r="C6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="15">
         <v>2E-3</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="15">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="15">
         <v>1.6E-2</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="15">
         <v>3.2800000000000003E-2</v>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="15">
         <v>4.0000000000000002E-4</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="15">
         <v>8.0000000000000004E-4</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J6" s="15">
         <v>2.8E-3</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="15">
         <v>6.9199999999999998E-2</v>
       </c>
-      <c r="L6" s="2">
-        <v>0</v>
-      </c>
-      <c r="M6" s="3">
+      <c r="L6" s="15">
+        <v>0</v>
+      </c>
+      <c r="M6" s="15">
         <v>5.1200000000000002E-2</v>
       </c>
-      <c r="N6" s="3">
+      <c r="N6" s="15">
         <v>0.61499999999999999</v>
       </c>
-      <c r="O6" s="3">
+      <c r="O6" s="15">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="P6" s="3">
+      <c r="P6" s="15">
         <v>0.01</v>
       </c>
     </row>
@@ -8053,43 +8054,43 @@
       <c r="C7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="2">
-        <v>0</v>
-      </c>
-      <c r="E7" s="2">
-        <v>0</v>
-      </c>
-      <c r="F7" s="2">
-        <v>0</v>
-      </c>
-      <c r="G7" s="2">
-        <v>0</v>
-      </c>
-      <c r="H7" s="2">
-        <v>0</v>
-      </c>
-      <c r="I7" s="2">
-        <v>0</v>
-      </c>
-      <c r="J7" s="2">
-        <v>0</v>
-      </c>
-      <c r="K7" s="2">
-        <v>0</v>
-      </c>
-      <c r="L7" s="2">
-        <v>0</v>
-      </c>
-      <c r="M7" s="3">
+      <c r="D7" s="15">
+        <v>0</v>
+      </c>
+      <c r="E7" s="15">
+        <v>0</v>
+      </c>
+      <c r="F7" s="15">
+        <v>0</v>
+      </c>
+      <c r="G7" s="15">
+        <v>0</v>
+      </c>
+      <c r="H7" s="15">
+        <v>0</v>
+      </c>
+      <c r="I7" s="15">
+        <v>0</v>
+      </c>
+      <c r="J7" s="15">
+        <v>0</v>
+      </c>
+      <c r="K7" s="15">
+        <v>0</v>
+      </c>
+      <c r="L7" s="15">
+        <v>0</v>
+      </c>
+      <c r="M7" s="15">
         <v>0.997</v>
       </c>
-      <c r="N7" s="2">
-        <v>0</v>
-      </c>
-      <c r="O7" s="2">
-        <v>0</v>
-      </c>
-      <c r="P7" s="2">
+      <c r="N7" s="15">
+        <v>0</v>
+      </c>
+      <c r="O7" s="15">
+        <v>0</v>
+      </c>
+      <c r="P7" s="15">
         <v>0</v>
       </c>
     </row>
@@ -8100,43 +8101,43 @@
       <c r="C8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="2">
-        <v>0</v>
-      </c>
-      <c r="E8" s="2">
-        <v>0</v>
-      </c>
-      <c r="F8" s="2">
-        <v>0</v>
-      </c>
-      <c r="G8" s="2">
-        <v>0</v>
-      </c>
-      <c r="H8" s="2">
-        <v>0</v>
-      </c>
-      <c r="I8" s="2">
-        <v>0</v>
-      </c>
-      <c r="J8" s="2">
-        <v>0</v>
-      </c>
-      <c r="K8" s="2">
-        <v>0</v>
-      </c>
-      <c r="L8" s="2">
-        <v>0</v>
-      </c>
-      <c r="M8" s="3">
+      <c r="D8" s="15">
+        <v>0</v>
+      </c>
+      <c r="E8" s="15">
+        <v>0</v>
+      </c>
+      <c r="F8" s="15">
+        <v>0</v>
+      </c>
+      <c r="G8" s="15">
+        <v>0</v>
+      </c>
+      <c r="H8" s="15">
+        <v>0</v>
+      </c>
+      <c r="I8" s="15">
+        <v>0</v>
+      </c>
+      <c r="J8" s="15">
+        <v>0</v>
+      </c>
+      <c r="K8" s="15">
+        <v>0</v>
+      </c>
+      <c r="L8" s="15">
+        <v>0</v>
+      </c>
+      <c r="M8" s="15">
         <v>0.996</v>
       </c>
-      <c r="N8" s="3">
+      <c r="N8" s="15">
         <v>4.3E-3</v>
       </c>
-      <c r="O8" s="2">
-        <v>0</v>
-      </c>
-      <c r="P8" s="2">
+      <c r="O8" s="15">
+        <v>0</v>
+      </c>
+      <c r="P8" s="15">
         <v>0</v>
       </c>
     </row>
@@ -8147,43 +8148,43 @@
       <c r="C9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="15">
         <v>5.7000000000000002E-3</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="15">
         <v>0.11</v>
       </c>
-      <c r="F9" s="2">
-        <v>0</v>
-      </c>
-      <c r="G9" s="3">
+      <c r="F9" s="15">
+        <v>0</v>
+      </c>
+      <c r="G9" s="15">
         <v>3.5499999999999997E-2</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="15">
         <v>4.5999999999999999E-3</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="15">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="J9" s="2">
-        <v>0</v>
-      </c>
-      <c r="K9" s="3">
+      <c r="J9" s="15">
+        <v>0</v>
+      </c>
+      <c r="K9" s="15">
         <v>7.3200000000000001E-2</v>
       </c>
-      <c r="L9" s="2">
-        <v>0</v>
-      </c>
-      <c r="M9" s="3">
+      <c r="L9" s="15">
+        <v>0</v>
+      </c>
+      <c r="M9" s="15">
         <v>3.78E-2</v>
       </c>
-      <c r="N9" s="3">
+      <c r="N9" s="15">
         <v>7.0900000000000005E-2</v>
       </c>
-      <c r="O9" s="3">
+      <c r="O9" s="15">
         <v>3.3999999999999998E-3</v>
       </c>
-      <c r="P9" s="3">
+      <c r="P9" s="15">
         <v>1.1000000000000001E-3</v>
       </c>
     </row>
@@ -8194,43 +8195,43 @@
       <c r="C10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="15">
         <v>6.6E-3</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="15">
         <v>9.9599999999999994E-2</v>
       </c>
-      <c r="F10" s="2">
-        <v>0</v>
-      </c>
-      <c r="G10" s="3">
+      <c r="F10" s="15">
+        <v>0</v>
+      </c>
+      <c r="G10" s="15">
         <v>4.6199999999999998E-2</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="15">
         <v>4.1000000000000003E-3</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="15">
         <v>1E-3</v>
       </c>
-      <c r="J10" s="2">
-        <v>0</v>
-      </c>
-      <c r="K10" s="3">
+      <c r="J10" s="15">
+        <v>0</v>
+      </c>
+      <c r="K10" s="15">
         <v>8.1799999999999998E-2</v>
       </c>
-      <c r="L10" s="2">
-        <v>0</v>
-      </c>
-      <c r="M10" s="3">
+      <c r="L10" s="15">
+        <v>0</v>
+      </c>
+      <c r="M10" s="15">
         <v>4.9299999999999997E-2</v>
       </c>
-      <c r="N10" s="3">
+      <c r="N10" s="15">
         <v>8.3799999999999999E-2</v>
       </c>
-      <c r="O10" s="3">
+      <c r="O10" s="15">
         <v>2E-3</v>
       </c>
-      <c r="P10" s="3">
+      <c r="P10" s="15">
         <v>5.5999999999999999E-3</v>
       </c>
     </row>
@@ -8241,43 +8242,43 @@
       <c r="C11" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="15">
         <v>5.7000000000000002E-3</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="15">
         <v>0.11</v>
       </c>
-      <c r="F11" s="2">
-        <v>0</v>
-      </c>
-      <c r="G11" s="3">
+      <c r="F11" s="15">
+        <v>0</v>
+      </c>
+      <c r="G11" s="15">
         <v>3.5499999999999997E-2</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="15">
         <v>4.5999999999999999E-3</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="15">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="J11" s="2">
-        <v>0</v>
-      </c>
-      <c r="K11" s="3">
+      <c r="J11" s="15">
+        <v>0</v>
+      </c>
+      <c r="K11" s="15">
         <v>7.3200000000000001E-2</v>
       </c>
-      <c r="L11" s="2">
-        <v>0</v>
-      </c>
-      <c r="M11" s="3">
+      <c r="L11" s="15">
+        <v>0</v>
+      </c>
+      <c r="M11" s="15">
         <v>3.78E-2</v>
       </c>
-      <c r="N11" s="3">
+      <c r="N11" s="15">
         <v>7.0900000000000005E-2</v>
       </c>
-      <c r="O11" s="3">
+      <c r="O11" s="15">
         <v>3.3999999999999998E-3</v>
       </c>
-      <c r="P11" s="3">
+      <c r="P11" s="15">
         <v>1.1000000000000001E-3</v>
       </c>
     </row>
@@ -8288,43 +8289,43 @@
       <c r="C12" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="15">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="15">
         <v>3.8699999999999998E-2</v>
       </c>
-      <c r="F12" s="2">
-        <v>0</v>
-      </c>
-      <c r="G12" s="3">
+      <c r="F12" s="15">
+        <v>0</v>
+      </c>
+      <c r="G12" s="15">
         <v>3.5499999999999997E-2</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="15">
         <v>7.9000000000000001E-4</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="15">
         <v>7.9000000000000001E-4</v>
       </c>
-      <c r="J12" s="2">
-        <v>0</v>
-      </c>
-      <c r="K12" s="3">
+      <c r="J12" s="15">
+        <v>0</v>
+      </c>
+      <c r="K12" s="15">
         <v>9.4E-2</v>
       </c>
-      <c r="L12" s="2">
-        <v>0</v>
-      </c>
-      <c r="M12" s="3">
+      <c r="L12" s="15">
+        <v>0</v>
+      </c>
+      <c r="M12" s="15">
         <v>5.21E-2</v>
       </c>
-      <c r="N12" s="3">
+      <c r="N12" s="15">
         <v>7.1099999999999997E-2</v>
       </c>
-      <c r="O12" s="3">
+      <c r="O12" s="15">
         <v>7.9000000000000001E-4</v>
       </c>
-      <c r="P12" s="3">
+      <c r="P12" s="15">
         <v>3.2000000000000002E-3</v>
       </c>
     </row>
@@ -8335,43 +8336,43 @@
       <c r="C13" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="15">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="15">
         <v>3.8699999999999998E-2</v>
       </c>
-      <c r="F13" s="2">
-        <v>0</v>
-      </c>
-      <c r="G13" s="3">
+      <c r="F13" s="15">
+        <v>0</v>
+      </c>
+      <c r="G13" s="15">
         <v>3.5499999999999997E-2</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="15">
         <v>7.9000000000000001E-4</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="15">
         <v>7.9000000000000001E-4</v>
       </c>
-      <c r="J13" s="2">
-        <v>0</v>
-      </c>
-      <c r="K13" s="3">
+      <c r="J13" s="15">
+        <v>0</v>
+      </c>
+      <c r="K13" s="15">
         <v>9.4E-2</v>
       </c>
-      <c r="L13" s="2">
-        <v>0</v>
-      </c>
-      <c r="M13" s="3">
+      <c r="L13" s="15">
+        <v>0</v>
+      </c>
+      <c r="M13" s="15">
         <v>5.21E-2</v>
       </c>
-      <c r="N13" s="3">
+      <c r="N13" s="15">
         <v>7.1099999999999997E-2</v>
       </c>
-      <c r="O13" s="3">
+      <c r="O13" s="15">
         <v>7.9000000000000001E-4</v>
       </c>
-      <c r="P13" s="3">
+      <c r="P13" s="15">
         <v>3.2000000000000002E-3</v>
       </c>
     </row>
@@ -8382,43 +8383,43 @@
       <c r="C14" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="15">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="15">
         <v>3.5200000000000002E-2</v>
       </c>
-      <c r="F14" s="2">
-        <v>0</v>
-      </c>
-      <c r="G14" s="3">
+      <c r="F14" s="15">
+        <v>0</v>
+      </c>
+      <c r="G14" s="15">
         <v>4.6600000000000003E-2</v>
       </c>
-      <c r="H14" s="2">
-        <v>0</v>
-      </c>
-      <c r="I14" s="3">
+      <c r="H14" s="15">
+        <v>0</v>
+      </c>
+      <c r="I14" s="15">
         <v>1.2999999999999999E-3</v>
       </c>
-      <c r="J14" s="2">
-        <v>0</v>
-      </c>
-      <c r="K14" s="3">
+      <c r="J14" s="15">
+        <v>0</v>
+      </c>
+      <c r="K14" s="15">
         <v>0.13700000000000001</v>
       </c>
-      <c r="L14" s="2">
-        <v>0</v>
-      </c>
-      <c r="M14" s="3">
+      <c r="L14" s="15">
+        <v>0</v>
+      </c>
+      <c r="M14" s="15">
         <v>4.9099999999999998E-2</v>
       </c>
-      <c r="N14" s="3">
+      <c r="N14" s="15">
         <v>9.5699999999999993E-2</v>
       </c>
-      <c r="O14" s="3">
+      <c r="O14" s="15">
         <v>6.3000000000000003E-4</v>
       </c>
-      <c r="P14" s="3">
+      <c r="P14" s="15">
         <v>3.8E-3</v>
       </c>
     </row>
@@ -8429,43 +8430,43 @@
       <c r="C15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="2">
-        <v>0</v>
-      </c>
-      <c r="E15" s="2">
-        <v>0</v>
-      </c>
-      <c r="F15" s="2">
-        <v>0</v>
-      </c>
-      <c r="G15" s="2">
-        <v>0</v>
-      </c>
-      <c r="H15" s="2">
-        <v>0</v>
-      </c>
-      <c r="I15" s="2">
-        <v>0</v>
-      </c>
-      <c r="J15" s="2">
-        <v>0</v>
-      </c>
-      <c r="K15" s="2">
-        <v>0</v>
-      </c>
-      <c r="L15" s="2">
-        <v>0</v>
-      </c>
-      <c r="M15" s="3">
+      <c r="D15" s="15">
+        <v>0</v>
+      </c>
+      <c r="E15" s="15">
+        <v>0</v>
+      </c>
+      <c r="F15" s="15">
+        <v>0</v>
+      </c>
+      <c r="G15" s="15">
+        <v>0</v>
+      </c>
+      <c r="H15" s="15">
+        <v>0</v>
+      </c>
+      <c r="I15" s="15">
+        <v>0</v>
+      </c>
+      <c r="J15" s="15">
+        <v>0</v>
+      </c>
+      <c r="K15" s="15">
+        <v>0</v>
+      </c>
+      <c r="L15" s="15">
+        <v>0</v>
+      </c>
+      <c r="M15" s="15">
         <v>0.997</v>
       </c>
-      <c r="N15" s="2">
-        <v>0</v>
-      </c>
-      <c r="O15" s="2">
-        <v>0</v>
-      </c>
-      <c r="P15" s="2">
+      <c r="N15" s="15">
+        <v>0</v>
+      </c>
+      <c r="O15" s="15">
+        <v>0</v>
+      </c>
+      <c r="P15" s="15">
         <v>0</v>
       </c>
     </row>
@@ -8476,43 +8477,43 @@
       <c r="C16" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="2">
-        <v>0</v>
-      </c>
-      <c r="E16" s="3">
+      <c r="D16" s="15">
+        <v>0</v>
+      </c>
+      <c r="E16" s="15">
         <v>8.0600000000000005E-2</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="15">
         <v>2.1100000000000001E-2</v>
       </c>
-      <c r="G16" s="3">
+      <c r="G16" s="15">
         <v>0.26100000000000001</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="15">
         <v>4.3E-3</v>
       </c>
-      <c r="I16" s="3">
+      <c r="I16" s="15">
         <v>9.3000000000000005E-4</v>
       </c>
-      <c r="J16" s="3">
+      <c r="J16" s="15">
         <v>3.1E-4</v>
       </c>
-      <c r="K16" s="3">
+      <c r="K16" s="15">
         <v>3.9399999999999998E-2</v>
       </c>
-      <c r="L16" s="2">
-        <v>0</v>
-      </c>
-      <c r="M16" s="3">
+      <c r="L16" s="15">
+        <v>0</v>
+      </c>
+      <c r="M16" s="15">
         <v>0.15</v>
       </c>
-      <c r="N16" s="3">
+      <c r="N16" s="15">
         <v>0.21199999999999999</v>
       </c>
-      <c r="O16" s="3">
+      <c r="O16" s="15">
         <v>6.2E-4</v>
       </c>
-      <c r="P16" s="3">
+      <c r="P16" s="15">
         <v>6.4999999999999997E-3</v>
       </c>
     </row>
@@ -8523,43 +8524,43 @@
       <c r="C17" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="2">
-        <v>0</v>
-      </c>
-      <c r="E17" s="3">
+      <c r="D17" s="15">
+        <v>0</v>
+      </c>
+      <c r="E17" s="15">
         <v>0.222</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="15">
         <v>2.8400000000000002E-2</v>
       </c>
-      <c r="G17" s="3">
+      <c r="G17" s="15">
         <v>0.21299999999999999</v>
       </c>
-      <c r="H17" s="3">
+      <c r="H17" s="15">
         <v>4.3499999999999997E-2</v>
       </c>
-      <c r="I17" s="2">
-        <v>0</v>
-      </c>
-      <c r="J17" s="3">
+      <c r="I17" s="15">
+        <v>0</v>
+      </c>
+      <c r="J17" s="15">
         <v>9.5E-4</v>
       </c>
-      <c r="K17" s="3">
+      <c r="K17" s="15">
         <v>4.6399999999999997E-2</v>
       </c>
-      <c r="L17" s="2">
-        <v>0</v>
-      </c>
-      <c r="M17" s="3">
+      <c r="L17" s="15">
+        <v>0</v>
+      </c>
+      <c r="M17" s="15">
         <v>8.5099999999999995E-2</v>
       </c>
-      <c r="N17" s="3">
+      <c r="N17" s="15">
         <v>0.186</v>
       </c>
-      <c r="O17" s="3">
+      <c r="O17" s="15">
         <v>1.9E-3</v>
       </c>
-      <c r="P17" s="3">
+      <c r="P17" s="15">
         <v>6.6E-3</v>
       </c>
     </row>
@@ -8570,43 +8571,43 @@
       <c r="C18" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="2">
-        <v>0</v>
-      </c>
-      <c r="E18" s="3">
+      <c r="D18" s="15">
+        <v>0</v>
+      </c>
+      <c r="E18" s="15">
         <v>0.127</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="15">
         <v>2.18E-2</v>
       </c>
-      <c r="G18" s="3">
+      <c r="G18" s="15">
         <v>0.214</v>
       </c>
-      <c r="H18" s="3">
+      <c r="H18" s="15">
         <v>7.3000000000000001E-3</v>
       </c>
-      <c r="I18" s="2">
-        <v>0</v>
-      </c>
-      <c r="J18" s="3">
+      <c r="I18" s="15">
+        <v>0</v>
+      </c>
+      <c r="J18" s="15">
         <v>3.6000000000000002E-4</v>
       </c>
-      <c r="K18" s="3">
+      <c r="K18" s="15">
         <v>6.1199999999999997E-2</v>
       </c>
-      <c r="L18" s="2">
-        <v>0</v>
-      </c>
-      <c r="M18" s="3">
+      <c r="L18" s="15">
+        <v>0</v>
+      </c>
+      <c r="M18" s="15">
         <v>0.16800000000000001</v>
       </c>
-      <c r="N18" s="3">
+      <c r="N18" s="15">
         <v>0.245</v>
       </c>
-      <c r="O18" s="3">
+      <c r="O18" s="15">
         <v>1.5E-3</v>
       </c>
-      <c r="P18" s="3">
+      <c r="P18" s="15">
         <v>1.0200000000000001E-2</v>
       </c>
     </row>
@@ -8617,43 +8618,43 @@
       <c r="C19" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="2">
-        <v>0</v>
-      </c>
-      <c r="E19" s="3">
+      <c r="D19" s="15">
+        <v>0</v>
+      </c>
+      <c r="E19" s="15">
         <v>2.35E-2</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="15">
         <v>1.1299999999999999E-2</v>
       </c>
-      <c r="G19" s="3">
+      <c r="G19" s="15">
         <v>0.14799999999999999</v>
       </c>
-      <c r="H19" s="3">
+      <c r="H19" s="15">
         <v>4.4999999999999999E-4</v>
       </c>
-      <c r="I19" s="2">
-        <v>0</v>
-      </c>
-      <c r="J19" s="2">
-        <v>0</v>
-      </c>
-      <c r="K19" s="3">
+      <c r="I19" s="15">
+        <v>0</v>
+      </c>
+      <c r="J19" s="15">
+        <v>0</v>
+      </c>
+      <c r="K19" s="15">
         <v>9.0899999999999995E-2</v>
       </c>
-      <c r="L19" s="2">
-        <v>0</v>
-      </c>
-      <c r="M19" s="3">
+      <c r="L19" s="15">
+        <v>0</v>
+      </c>
+      <c r="M19" s="15">
         <v>0.19800000000000001</v>
       </c>
-      <c r="N19" s="3">
+      <c r="N19" s="15">
         <v>0.27100000000000002</v>
       </c>
-      <c r="O19" s="3">
+      <c r="O19" s="15">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="P19" s="3">
+      <c r="P19" s="15">
         <v>3.5999999999999999E-3</v>
       </c>
     </row>
@@ -8664,43 +8665,43 @@
       <c r="C20" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D20" s="2">
-        <v>0</v>
-      </c>
-      <c r="E20" s="3">
+      <c r="D20" s="15">
+        <v>0</v>
+      </c>
+      <c r="E20" s="15">
         <v>0.113</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="15">
         <v>3.0499999999999999E-2</v>
       </c>
-      <c r="G20" s="3">
+      <c r="G20" s="15">
         <v>0.20200000000000001</v>
       </c>
-      <c r="H20" s="3">
+      <c r="H20" s="15">
         <v>3.1800000000000002E-2</v>
       </c>
-      <c r="I20" s="2">
-        <v>0</v>
-      </c>
-      <c r="J20" s="2">
-        <v>0</v>
-      </c>
-      <c r="K20" s="3">
+      <c r="I20" s="15">
+        <v>0</v>
+      </c>
+      <c r="J20" s="15">
+        <v>0</v>
+      </c>
+      <c r="K20" s="15">
         <v>5.9700000000000003E-2</v>
       </c>
-      <c r="L20" s="2">
-        <v>0</v>
-      </c>
-      <c r="M20" s="3">
+      <c r="L20" s="15">
+        <v>0</v>
+      </c>
+      <c r="M20" s="15">
         <v>0.123</v>
       </c>
-      <c r="N20" s="3">
+      <c r="N20" s="15">
         <v>0.24399999999999999</v>
       </c>
-      <c r="O20" s="2">
-        <v>0</v>
-      </c>
-      <c r="P20" s="3">
+      <c r="O20" s="15">
+        <v>0</v>
+      </c>
+      <c r="P20" s="15">
         <v>5.3E-3</v>
       </c>
     </row>
@@ -8711,43 +8712,43 @@
       <c r="C21" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="2">
-        <v>0</v>
-      </c>
-      <c r="E21" s="3">
+      <c r="D21" s="15">
+        <v>0</v>
+      </c>
+      <c r="E21" s="15">
         <v>1.6299999999999999E-2</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="15">
         <v>1.6299999999999999E-2</v>
       </c>
-      <c r="G21" s="3">
+      <c r="G21" s="15">
         <v>0.16600000000000001</v>
       </c>
-      <c r="H21" s="3">
+      <c r="H21" s="15">
         <v>8.5999999999999998E-4</v>
       </c>
-      <c r="I21" s="2">
-        <v>0</v>
-      </c>
-      <c r="J21" s="3">
+      <c r="I21" s="15">
+        <v>0</v>
+      </c>
+      <c r="J21" s="15">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="K21" s="3">
+      <c r="K21" s="15">
         <v>6.7500000000000004E-2</v>
       </c>
-      <c r="L21" s="3">
+      <c r="L21" s="15">
         <v>4.2999999999999999E-4</v>
       </c>
-      <c r="M21" s="3">
+      <c r="M21" s="15">
         <v>0.19700000000000001</v>
       </c>
-      <c r="N21" s="3">
+      <c r="N21" s="15">
         <v>0.32700000000000001</v>
       </c>
-      <c r="O21" s="3">
+      <c r="O21" s="15">
         <v>1.2999999999999999E-3</v>
       </c>
-      <c r="P21" s="3">
+      <c r="P21" s="15">
         <v>4.3E-3</v>
       </c>
     </row>
@@ -8758,43 +8759,43 @@
       <c r="C22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="2">
-        <v>0</v>
-      </c>
-      <c r="E22" s="2">
-        <v>0</v>
-      </c>
-      <c r="F22" s="2">
-        <v>0</v>
-      </c>
-      <c r="G22" s="2">
-        <v>0</v>
-      </c>
-      <c r="H22" s="2">
-        <v>0</v>
-      </c>
-      <c r="I22" s="2">
-        <v>0</v>
-      </c>
-      <c r="J22" s="2">
-        <v>0</v>
-      </c>
-      <c r="K22" s="2">
-        <v>0</v>
-      </c>
-      <c r="L22" s="2">
-        <v>0</v>
-      </c>
-      <c r="M22" s="3">
+      <c r="D22" s="15">
+        <v>0</v>
+      </c>
+      <c r="E22" s="15">
+        <v>0</v>
+      </c>
+      <c r="F22" s="15">
+        <v>0</v>
+      </c>
+      <c r="G22" s="15">
+        <v>0</v>
+      </c>
+      <c r="H22" s="15">
+        <v>0</v>
+      </c>
+      <c r="I22" s="15">
+        <v>0</v>
+      </c>
+      <c r="J22" s="15">
+        <v>0</v>
+      </c>
+      <c r="K22" s="15">
+        <v>0</v>
+      </c>
+      <c r="L22" s="15">
+        <v>0</v>
+      </c>
+      <c r="M22" s="15">
         <v>0.99199999999999999</v>
       </c>
-      <c r="N22" s="3">
+      <c r="N22" s="15">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="O22" s="2">
-        <v>0</v>
-      </c>
-      <c r="P22" s="2">
+      <c r="O22" s="15">
+        <v>0</v>
+      </c>
+      <c r="P22" s="15">
         <v>0</v>
       </c>
     </row>
@@ -8805,43 +8806,43 @@
       <c r="C23" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D23" s="2">
-        <v>0</v>
-      </c>
-      <c r="E23" s="3">
+      <c r="D23" s="15">
+        <v>0</v>
+      </c>
+      <c r="E23" s="15">
         <v>1.5E-3</v>
       </c>
-      <c r="F23" s="3">
+      <c r="F23" s="15">
         <v>6.4999999999999997E-3</v>
       </c>
-      <c r="G23" s="3">
+      <c r="G23" s="15">
         <v>9.4100000000000003E-2</v>
       </c>
-      <c r="H23" s="2">
-        <v>0</v>
-      </c>
-      <c r="I23" s="2">
-        <v>0</v>
-      </c>
-      <c r="J23" s="3">
+      <c r="H23" s="15">
+        <v>0</v>
+      </c>
+      <c r="I23" s="15">
+        <v>0</v>
+      </c>
+      <c r="J23" s="15">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="K23" s="3">
+      <c r="K23" s="15">
         <v>0.111</v>
       </c>
-      <c r="L23" s="2">
-        <v>0</v>
-      </c>
-      <c r="M23" s="3">
+      <c r="L23" s="15">
+        <v>0</v>
+      </c>
+      <c r="M23" s="15">
         <v>0.28499999999999998</v>
       </c>
-      <c r="N23" s="3">
+      <c r="N23" s="15">
         <v>0.32</v>
       </c>
-      <c r="O23" s="3">
+      <c r="O23" s="15">
         <v>2.3E-3</v>
       </c>
-      <c r="P23" s="3">
+      <c r="P23" s="15">
         <v>3.15E-2</v>
       </c>
     </row>
@@ -8852,43 +8853,43 @@
       <c r="C24" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D24" s="2">
-        <v>0</v>
-      </c>
-      <c r="E24" s="2">
-        <v>0</v>
-      </c>
-      <c r="F24" s="3">
+      <c r="D24" s="15">
+        <v>0</v>
+      </c>
+      <c r="E24" s="15">
+        <v>0</v>
+      </c>
+      <c r="F24" s="15">
         <v>0.01</v>
       </c>
-      <c r="G24" s="3">
+      <c r="G24" s="15">
         <v>0.13100000000000001</v>
       </c>
-      <c r="H24" s="2">
-        <v>0</v>
-      </c>
-      <c r="I24" s="2">
-        <v>0</v>
-      </c>
-      <c r="J24" s="3">
+      <c r="H24" s="15">
+        <v>0</v>
+      </c>
+      <c r="I24" s="15">
+        <v>0</v>
+      </c>
+      <c r="J24" s="15">
         <v>3.8E-3</v>
       </c>
-      <c r="K24" s="3">
+      <c r="K24" s="15">
         <v>0.129</v>
       </c>
-      <c r="L24" s="2">
-        <v>0</v>
-      </c>
-      <c r="M24" s="3">
+      <c r="L24" s="15">
+        <v>0</v>
+      </c>
+      <c r="M24" s="15">
         <v>0.128</v>
       </c>
-      <c r="N24" s="3">
+      <c r="N24" s="15">
         <v>0.40100000000000002</v>
       </c>
-      <c r="O24" s="3">
+      <c r="O24" s="15">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="P24" s="3">
+      <c r="P24" s="15">
         <v>2.12E-2</v>
       </c>
     </row>
@@ -8899,43 +8900,43 @@
       <c r="C25" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D25" s="2">
-        <v>0</v>
-      </c>
-      <c r="E25" s="3">
+      <c r="D25" s="15">
+        <v>0</v>
+      </c>
+      <c r="E25" s="15">
         <v>3.4000000000000002E-4</v>
       </c>
-      <c r="F25" s="3">
+      <c r="F25" s="15">
         <v>7.7999999999999996E-3</v>
       </c>
-      <c r="G25" s="3">
+      <c r="G25" s="15">
         <v>8.8200000000000001E-2</v>
       </c>
-      <c r="H25" s="2">
-        <v>0</v>
-      </c>
-      <c r="I25" s="3">
+      <c r="H25" s="15">
+        <v>0</v>
+      </c>
+      <c r="I25" s="15">
         <v>3.4000000000000002E-4</v>
       </c>
-      <c r="J25" s="3">
+      <c r="J25" s="15">
         <v>1E-3</v>
       </c>
-      <c r="K25" s="3">
+      <c r="K25" s="15">
         <v>0.129</v>
       </c>
-      <c r="L25" s="2">
-        <v>0</v>
-      </c>
-      <c r="M25" s="3">
+      <c r="L25" s="15">
+        <v>0</v>
+      </c>
+      <c r="M25" s="15">
         <v>0.27600000000000002</v>
       </c>
-      <c r="N25" s="3">
+      <c r="N25" s="15">
         <v>0.35399999999999998</v>
       </c>
-      <c r="O25" s="3">
+      <c r="O25" s="15">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="P25" s="3">
+      <c r="P25" s="15">
         <v>4.24E-2</v>
       </c>
     </row>
@@ -8946,43 +8947,43 @@
       <c r="C26" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D26" s="2">
-        <v>0</v>
-      </c>
-      <c r="E26" s="2">
-        <v>0</v>
-      </c>
-      <c r="F26" s="3">
+      <c r="D26" s="15">
+        <v>0</v>
+      </c>
+      <c r="E26" s="15">
+        <v>0</v>
+      </c>
+      <c r="F26" s="15">
         <v>6.4000000000000003E-3</v>
       </c>
-      <c r="G26" s="3">
+      <c r="G26" s="15">
         <v>4.2999999999999997E-2</v>
       </c>
-      <c r="H26" s="2">
-        <v>0</v>
-      </c>
-      <c r="I26" s="2">
-        <v>0</v>
-      </c>
-      <c r="J26" s="3">
+      <c r="H26" s="15">
+        <v>0</v>
+      </c>
+      <c r="I26" s="15">
+        <v>0</v>
+      </c>
+      <c r="J26" s="15">
         <v>3.8E-3</v>
       </c>
-      <c r="K26" s="3">
+      <c r="K26" s="15">
         <v>0.16400000000000001</v>
       </c>
-      <c r="L26" s="2">
-        <v>0</v>
-      </c>
-      <c r="M26" s="3">
+      <c r="L26" s="15">
+        <v>0</v>
+      </c>
+      <c r="M26" s="15">
         <v>0.30099999999999999</v>
       </c>
-      <c r="N26" s="3">
+      <c r="N26" s="15">
         <v>0.32700000000000001</v>
       </c>
-      <c r="O26" s="3">
+      <c r="O26" s="15">
         <v>4.4999999999999997E-3</v>
       </c>
-      <c r="P26" s="3">
+      <c r="P26" s="15">
         <v>1.3599999999999999E-2</v>
       </c>
     </row>
@@ -8993,43 +8994,43 @@
       <c r="C27" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D27" s="2">
-        <v>0</v>
-      </c>
-      <c r="E27" s="2">
-        <v>0</v>
-      </c>
-      <c r="F27" s="3">
+      <c r="D27" s="15">
+        <v>0</v>
+      </c>
+      <c r="E27" s="15">
+        <v>0</v>
+      </c>
+      <c r="F27" s="15">
         <v>8.2000000000000007E-3</v>
       </c>
-      <c r="G27" s="3">
+      <c r="G27" s="15">
         <v>0.17</v>
       </c>
-      <c r="H27" s="2">
-        <v>0</v>
-      </c>
-      <c r="I27" s="2">
-        <v>0</v>
-      </c>
-      <c r="J27" s="3">
+      <c r="H27" s="15">
+        <v>0</v>
+      </c>
+      <c r="I27" s="15">
+        <v>0</v>
+      </c>
+      <c r="J27" s="15">
         <v>8.2000000000000007E-3</v>
       </c>
-      <c r="K27" s="3">
+      <c r="K27" s="15">
         <v>0.16</v>
       </c>
-      <c r="L27" s="2">
-        <v>0</v>
-      </c>
-      <c r="M27" s="3">
+      <c r="L27" s="15">
+        <v>0</v>
+      </c>
+      <c r="M27" s="15">
         <v>0.18099999999999999</v>
       </c>
-      <c r="N27" s="3">
+      <c r="N27" s="15">
         <v>0.28100000000000003</v>
       </c>
-      <c r="O27" s="3">
+      <c r="O27" s="15">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="P27" s="3">
+      <c r="P27" s="15">
         <v>2.58E-2</v>
       </c>
     </row>
@@ -9040,43 +9041,43 @@
       <c r="C28" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="2">
-        <v>0</v>
-      </c>
-      <c r="E28" s="2">
-        <v>0</v>
-      </c>
-      <c r="F28" s="3">
+      <c r="D28" s="15">
+        <v>0</v>
+      </c>
+      <c r="E28" s="15">
+        <v>0</v>
+      </c>
+      <c r="F28" s="15">
         <v>4.4999999999999997E-3</v>
       </c>
-      <c r="G28" s="3">
+      <c r="G28" s="15">
         <v>5.5399999999999998E-2</v>
       </c>
-      <c r="H28" s="2">
-        <v>0</v>
-      </c>
-      <c r="I28" s="3">
+      <c r="H28" s="15">
+        <v>0</v>
+      </c>
+      <c r="I28" s="15">
         <v>3.2000000000000003E-4</v>
       </c>
-      <c r="J28" s="3">
+      <c r="J28" s="15">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="K28" s="3">
+      <c r="K28" s="15">
         <v>0.14799999999999999</v>
       </c>
-      <c r="L28" s="2">
-        <v>0</v>
-      </c>
-      <c r="M28" s="3">
+      <c r="L28" s="15">
+        <v>0</v>
+      </c>
+      <c r="M28" s="15">
         <v>0.316</v>
       </c>
-      <c r="N28" s="3">
+      <c r="N28" s="15">
         <v>0.35399999999999998</v>
       </c>
-      <c r="O28" s="3">
+      <c r="O28" s="15">
         <v>2.3E-3</v>
       </c>
-      <c r="P28" s="3">
+      <c r="P28" s="15">
         <v>1.8700000000000001E-2</v>
       </c>
     </row>
@@ -9087,43 +9088,43 @@
       <c r="C29" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="2">
-        <v>0</v>
-      </c>
-      <c r="E29" s="2">
-        <v>0</v>
-      </c>
-      <c r="F29" s="2">
-        <v>0</v>
-      </c>
-      <c r="G29" s="2">
-        <v>0</v>
-      </c>
-      <c r="H29" s="2">
-        <v>0</v>
-      </c>
-      <c r="I29" s="2">
-        <v>0</v>
-      </c>
-      <c r="J29" s="2">
-        <v>0</v>
-      </c>
-      <c r="K29" s="2">
-        <v>0</v>
-      </c>
-      <c r="L29" s="2">
-        <v>0</v>
-      </c>
-      <c r="M29" s="3">
+      <c r="D29" s="15">
+        <v>0</v>
+      </c>
+      <c r="E29" s="15">
+        <v>0</v>
+      </c>
+      <c r="F29" s="15">
+        <v>0</v>
+      </c>
+      <c r="G29" s="15">
+        <v>0</v>
+      </c>
+      <c r="H29" s="15">
+        <v>0</v>
+      </c>
+      <c r="I29" s="15">
+        <v>0</v>
+      </c>
+      <c r="J29" s="15">
+        <v>0</v>
+      </c>
+      <c r="K29" s="15">
+        <v>0</v>
+      </c>
+      <c r="L29" s="15">
+        <v>0</v>
+      </c>
+      <c r="M29" s="15">
         <v>0.98299999999999998</v>
       </c>
-      <c r="N29" s="2">
-        <v>0</v>
-      </c>
-      <c r="O29" s="2">
-        <v>0</v>
-      </c>
-      <c r="P29" s="2">
+      <c r="N29" s="15">
+        <v>0</v>
+      </c>
+      <c r="O29" s="15">
+        <v>0</v>
+      </c>
+      <c r="P29" s="15">
         <v>0</v>
       </c>
     </row>
@@ -9134,43 +9135,43 @@
       <c r="C30" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D30" s="2">
-        <v>0</v>
-      </c>
-      <c r="E30" s="3">
+      <c r="D30" s="15">
+        <v>0</v>
+      </c>
+      <c r="E30" s="15">
         <v>8.8000000000000005E-3</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30" s="15">
         <v>8.3999999999999995E-3</v>
       </c>
-      <c r="G30" s="3">
+      <c r="G30" s="15">
         <v>2.3699999999999999E-2</v>
       </c>
-      <c r="H30" s="3">
+      <c r="H30" s="15">
         <v>2E-3</v>
       </c>
-      <c r="I30" s="3">
+      <c r="I30" s="15">
         <v>3.5E-4</v>
       </c>
-      <c r="J30" s="3">
+      <c r="J30" s="15">
         <v>1.4E-3</v>
       </c>
-      <c r="K30" s="3">
+      <c r="K30" s="15">
         <v>0.16300000000000001</v>
       </c>
-      <c r="L30" s="3">
+      <c r="L30" s="15">
         <v>1.2E-4</v>
       </c>
-      <c r="M30" s="3">
+      <c r="M30" s="15">
         <v>0.432</v>
       </c>
-      <c r="N30" s="3">
+      <c r="N30" s="15">
         <v>0.153</v>
       </c>
-      <c r="O30" s="3">
+      <c r="O30" s="15">
         <v>1.2E-4</v>
       </c>
-      <c r="P30" s="3">
+      <c r="P30" s="15">
         <v>0.112</v>
       </c>
     </row>
@@ -9181,43 +9182,43 @@
       <c r="C31" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D31" s="2">
-        <v>0</v>
-      </c>
-      <c r="E31" s="3">
+      <c r="D31" s="15">
+        <v>0</v>
+      </c>
+      <c r="E31" s="15">
         <v>1.2699999999999999E-2</v>
       </c>
-      <c r="F31" s="3">
+      <c r="F31" s="15">
         <v>8.2000000000000007E-3</v>
       </c>
-      <c r="G31" s="3">
+      <c r="G31" s="15">
         <v>4.1000000000000002E-2</v>
       </c>
-      <c r="H31" s="3">
+      <c r="H31" s="15">
         <v>2.3E-3</v>
       </c>
-      <c r="I31" s="3">
+      <c r="I31" s="15">
         <v>4.6000000000000001E-4</v>
       </c>
-      <c r="J31" s="3">
+      <c r="J31" s="15">
         <v>4.6000000000000001E-4</v>
       </c>
-      <c r="K31" s="3">
+      <c r="K31" s="15">
         <v>0.17100000000000001</v>
       </c>
-      <c r="L31" s="2">
-        <v>0</v>
-      </c>
-      <c r="M31" s="3">
+      <c r="L31" s="15">
+        <v>0</v>
+      </c>
+      <c r="M31" s="15">
         <v>0.33200000000000002</v>
       </c>
-      <c r="N31" s="3">
+      <c r="N31" s="15">
         <v>0.18099999999999999</v>
       </c>
-      <c r="O31" s="2">
-        <v>0</v>
-      </c>
-      <c r="P31" s="3">
+      <c r="O31" s="15">
+        <v>0</v>
+      </c>
+      <c r="P31" s="15">
         <v>0.14399999999999999</v>
       </c>
     </row>
@@ -9228,43 +9229,43 @@
       <c r="C32" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D32" s="2">
-        <v>0</v>
-      </c>
-      <c r="E32" s="3">
+      <c r="D32" s="15">
+        <v>0</v>
+      </c>
+      <c r="E32" s="15">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="F32" s="3">
+      <c r="F32" s="15">
         <v>7.9000000000000008E-3</v>
       </c>
-      <c r="G32" s="3">
+      <c r="G32" s="15">
         <v>2.6700000000000002E-2</v>
       </c>
-      <c r="H32" s="3">
+      <c r="H32" s="15">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="I32" s="3">
+      <c r="I32" s="15">
         <v>2.2000000000000001E-4</v>
       </c>
-      <c r="J32" s="3">
+      <c r="J32" s="15">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="K32" s="3">
+      <c r="K32" s="15">
         <v>0.17699999999999999</v>
       </c>
-      <c r="L32" s="2">
-        <v>0</v>
-      </c>
-      <c r="M32" s="3">
+      <c r="L32" s="15">
+        <v>0</v>
+      </c>
+      <c r="M32" s="15">
         <v>0.35699999999999998</v>
       </c>
-      <c r="N32" s="3">
+      <c r="N32" s="15">
         <v>0.18099999999999999</v>
       </c>
-      <c r="O32" s="2">
-        <v>0</v>
-      </c>
-      <c r="P32" s="3">
+      <c r="O32" s="15">
+        <v>0</v>
+      </c>
+      <c r="P32" s="15">
         <v>0.16800000000000001</v>
       </c>
     </row>
@@ -9275,43 +9276,43 @@
       <c r="C33" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D33" s="2">
-        <v>0</v>
-      </c>
-      <c r="E33" s="3">
+      <c r="D33" s="15">
+        <v>0</v>
+      </c>
+      <c r="E33" s="15">
         <v>4.8000000000000001E-4</v>
       </c>
-      <c r="F33" s="3">
+      <c r="F33" s="15">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="G33" s="3">
+      <c r="G33" s="15">
         <v>1.3599999999999999E-2</v>
       </c>
-      <c r="H33" s="4">
+      <c r="H33" s="15">
         <v>9.5199999999999997E-5</v>
       </c>
-      <c r="I33" s="3">
+      <c r="I33" s="15">
         <v>2.9E-4</v>
       </c>
-      <c r="J33" s="3">
+      <c r="J33" s="15">
         <v>6.7000000000000002E-4</v>
       </c>
-      <c r="K33" s="3">
+      <c r="K33" s="15">
         <v>0.151</v>
       </c>
-      <c r="L33" s="2">
-        <v>0</v>
-      </c>
-      <c r="M33" s="3">
+      <c r="L33" s="15">
+        <v>0</v>
+      </c>
+      <c r="M33" s="15">
         <v>0.505</v>
       </c>
-      <c r="N33" s="3">
+      <c r="N33" s="15">
         <v>0.14499999999999999</v>
       </c>
-      <c r="O33" s="4">
+      <c r="O33" s="15">
         <v>9.5199999999999997E-5</v>
       </c>
-      <c r="P33" s="3">
+      <c r="P33" s="15">
         <v>6.88E-2</v>
       </c>
     </row>
@@ -9322,43 +9323,43 @@
       <c r="C34" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D34" s="2">
-        <v>0</v>
-      </c>
-      <c r="E34" s="3">
+      <c r="D34" s="15">
+        <v>0</v>
+      </c>
+      <c r="E34" s="15">
         <v>9.1000000000000004E-3</v>
       </c>
-      <c r="F34" s="3">
+      <c r="F34" s="15">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="G34" s="3">
+      <c r="G34" s="15">
         <v>2.8500000000000001E-2</v>
       </c>
-      <c r="H34" s="3">
+      <c r="H34" s="15">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="I34" s="3">
+      <c r="I34" s="15">
         <v>7.6000000000000004E-4</v>
       </c>
-      <c r="J34" s="3">
+      <c r="J34" s="15">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="K34" s="3">
+      <c r="K34" s="15">
         <v>0.13600000000000001</v>
       </c>
-      <c r="L34" s="2">
-        <v>0</v>
-      </c>
-      <c r="M34" s="3">
+      <c r="L34" s="15">
+        <v>0</v>
+      </c>
+      <c r="M34" s="15">
         <v>0.35299999999999998</v>
       </c>
-      <c r="N34" s="3">
+      <c r="N34" s="15">
         <v>0.18</v>
       </c>
-      <c r="O34" s="3">
+      <c r="O34" s="15">
         <v>3.8000000000000002E-4</v>
       </c>
-      <c r="P34" s="3">
+      <c r="P34" s="15">
         <v>0.158</v>
       </c>
     </row>
@@ -9369,43 +9370,43 @@
       <c r="C35" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D35" s="2">
-        <v>0</v>
-      </c>
-      <c r="E35" s="3">
+      <c r="D35" s="15">
+        <v>0</v>
+      </c>
+      <c r="E35" s="15">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="F35" s="3">
+      <c r="F35" s="15">
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="G35" s="3">
+      <c r="G35" s="15">
         <v>1.6799999999999999E-2</v>
       </c>
-      <c r="H35" s="3">
+      <c r="H35" s="15">
         <v>1.6000000000000001E-4</v>
       </c>
-      <c r="I35" s="4">
+      <c r="I35" s="15">
         <v>7.7899999999999996E-5</v>
       </c>
-      <c r="J35" s="3">
+      <c r="J35" s="15">
         <v>1.8E-3</v>
       </c>
-      <c r="K35" s="3">
+      <c r="K35" s="15">
         <v>0.154</v>
       </c>
-      <c r="L35" s="2">
-        <v>0</v>
-      </c>
-      <c r="M35" s="3">
+      <c r="L35" s="15">
+        <v>0</v>
+      </c>
+      <c r="M35" s="15">
         <v>0.40100000000000002</v>
       </c>
-      <c r="N35" s="3">
+      <c r="N35" s="15">
         <v>0.16800000000000001</v>
       </c>
-      <c r="O35" s="2">
-        <v>0</v>
-      </c>
-      <c r="P35" s="3">
+      <c r="O35" s="15">
+        <v>0</v>
+      </c>
+      <c r="P35" s="15">
         <v>0.16200000000000001</v>
       </c>
     </row>
@@ -9416,43 +9417,43 @@
       <c r="C36" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D36" s="2">
-        <v>0</v>
-      </c>
-      <c r="E36" s="2">
-        <v>0</v>
-      </c>
-      <c r="F36" s="2">
-        <v>0</v>
-      </c>
-      <c r="G36" s="2">
-        <v>0</v>
-      </c>
-      <c r="H36" s="2">
-        <v>0</v>
-      </c>
-      <c r="I36" s="2">
-        <v>0</v>
-      </c>
-      <c r="J36" s="2">
-        <v>0</v>
-      </c>
-      <c r="K36" s="2">
-        <v>0</v>
-      </c>
-      <c r="L36" s="2">
-        <v>0</v>
-      </c>
-      <c r="M36" s="3">
+      <c r="D36" s="15">
+        <v>0</v>
+      </c>
+      <c r="E36" s="15">
+        <v>0</v>
+      </c>
+      <c r="F36" s="15">
+        <v>0</v>
+      </c>
+      <c r="G36" s="15">
+        <v>0</v>
+      </c>
+      <c r="H36" s="15">
+        <v>0</v>
+      </c>
+      <c r="I36" s="15">
+        <v>0</v>
+      </c>
+      <c r="J36" s="15">
+        <v>0</v>
+      </c>
+      <c r="K36" s="15">
+        <v>0</v>
+      </c>
+      <c r="L36" s="15">
+        <v>0</v>
+      </c>
+      <c r="M36" s="15">
         <v>0.98599999999999999</v>
       </c>
-      <c r="N36" s="2">
-        <v>0</v>
-      </c>
-      <c r="O36" s="3">
+      <c r="N36" s="15">
+        <v>0</v>
+      </c>
+      <c r="O36" s="15">
         <v>1.4E-3</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="15">
         <v>0</v>
       </c>
     </row>
@@ -9463,43 +9464,43 @@
       <c r="C37" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D37" s="2">
-        <v>0</v>
-      </c>
-      <c r="E37" s="3">
+      <c r="D37" s="15">
+        <v>0</v>
+      </c>
+      <c r="E37" s="15">
         <v>4.1999999999999997E-3</v>
       </c>
-      <c r="F37" s="3">
+      <c r="F37" s="15">
         <v>5.1999999999999998E-3</v>
       </c>
-      <c r="G37" s="3">
+      <c r="G37" s="15">
         <v>4.9299999999999997E-2</v>
       </c>
-      <c r="H37" s="4">
+      <c r="H37" s="15">
         <v>9.7200000000000004E-5</v>
       </c>
-      <c r="I37" s="3">
+      <c r="I37" s="15">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="J37" s="3">
+      <c r="J37" s="15">
         <v>3.8999999999999998E-3</v>
       </c>
-      <c r="K37" s="3">
+      <c r="K37" s="15">
         <v>0.109</v>
       </c>
-      <c r="L37" s="2">
-        <v>0</v>
-      </c>
-      <c r="M37" s="3">
+      <c r="L37" s="15">
+        <v>0</v>
+      </c>
+      <c r="M37" s="15">
         <v>0.33600000000000002</v>
       </c>
-      <c r="N37" s="3">
+      <c r="N37" s="15">
         <v>4.82E-2</v>
       </c>
-      <c r="O37" s="3">
+      <c r="O37" s="15">
         <v>2.8E-3</v>
       </c>
-      <c r="P37" s="3">
+      <c r="P37" s="15">
         <v>0.34200000000000003</v>
       </c>
     </row>
@@ -9510,43 +9511,43 @@
       <c r="C38" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D38" s="2">
-        <v>0</v>
-      </c>
-      <c r="E38" s="3">
+      <c r="D38" s="15">
+        <v>0</v>
+      </c>
+      <c r="E38" s="15">
         <v>8.8000000000000005E-3</v>
       </c>
-      <c r="F38" s="3">
+      <c r="F38" s="15">
         <v>2.0400000000000001E-2</v>
       </c>
-      <c r="G38" s="3">
+      <c r="G38" s="15">
         <v>0.10100000000000001</v>
       </c>
-      <c r="H38" s="2">
-        <v>0</v>
-      </c>
-      <c r="I38" s="3">
+      <c r="H38" s="15">
+        <v>0</v>
+      </c>
+      <c r="I38" s="15">
         <v>1.2999999999999999E-3</v>
       </c>
-      <c r="J38" s="3">
+      <c r="J38" s="15">
         <v>5.7000000000000002E-3</v>
       </c>
-      <c r="K38" s="3">
+      <c r="K38" s="15">
         <v>9.1700000000000004E-2</v>
       </c>
-      <c r="L38" s="2">
-        <v>0</v>
-      </c>
-      <c r="M38" s="3">
+      <c r="L38" s="15">
+        <v>0</v>
+      </c>
+      <c r="M38" s="15">
         <v>0.20499999999999999</v>
       </c>
-      <c r="N38" s="3">
+      <c r="N38" s="15">
         <v>7.3800000000000004E-2</v>
       </c>
-      <c r="O38" s="3">
+      <c r="O38" s="15">
         <v>1.1599999999999999E-2</v>
       </c>
-      <c r="P38" s="3">
+      <c r="P38" s="15">
         <v>0.32</v>
       </c>
     </row>
@@ -9557,43 +9558,43 @@
       <c r="C39" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D39" s="2">
-        <v>0</v>
-      </c>
-      <c r="E39" s="3">
+      <c r="D39" s="15">
+        <v>0</v>
+      </c>
+      <c r="E39" s="15">
         <v>6.8999999999999999E-3</v>
       </c>
-      <c r="F39" s="3">
+      <c r="F39" s="15">
         <v>1.38E-2</v>
       </c>
-      <c r="G39" s="3">
+      <c r="G39" s="15">
         <v>6.8400000000000002E-2</v>
       </c>
-      <c r="H39" s="2">
-        <v>0</v>
-      </c>
-      <c r="I39" s="3">
+      <c r="H39" s="15">
+        <v>0</v>
+      </c>
+      <c r="I39" s="15">
         <v>4.2999999999999999E-4</v>
       </c>
-      <c r="J39" s="3">
+      <c r="J39" s="15">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="K39" s="3">
+      <c r="K39" s="15">
         <v>9.7500000000000003E-2</v>
       </c>
-      <c r="L39" s="2">
-        <v>0</v>
-      </c>
-      <c r="M39" s="3">
+      <c r="L39" s="15">
+        <v>0</v>
+      </c>
+      <c r="M39" s="15">
         <v>0.20599999999999999</v>
       </c>
-      <c r="N39" s="3">
+      <c r="N39" s="15">
         <v>3.9199999999999999E-2</v>
       </c>
-      <c r="O39" s="3">
+      <c r="O39" s="15">
         <v>4.7999999999999996E-3</v>
       </c>
-      <c r="P39" s="3">
+      <c r="P39" s="15">
         <v>0.45700000000000002</v>
       </c>
     </row>
@@ -9604,43 +9605,43 @@
       <c r="C40" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D40" s="2">
-        <v>0</v>
-      </c>
-      <c r="E40" s="3">
+      <c r="D40" s="15">
+        <v>0</v>
+      </c>
+      <c r="E40" s="15">
         <v>8.6E-3</v>
       </c>
-      <c r="F40" s="3">
+      <c r="F40" s="15">
         <v>1.7399999999999999E-2</v>
       </c>
-      <c r="G40" s="3">
+      <c r="G40" s="15">
         <v>8.4400000000000003E-2</v>
       </c>
-      <c r="H40" s="2">
-        <v>0</v>
-      </c>
-      <c r="I40" s="3">
+      <c r="H40" s="15">
+        <v>0</v>
+      </c>
+      <c r="I40" s="15">
         <v>5.9000000000000003E-4</v>
       </c>
-      <c r="J40" s="3">
+      <c r="J40" s="15">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="K40" s="3">
+      <c r="K40" s="15">
         <v>9.01E-2</v>
       </c>
-      <c r="L40" s="2">
-        <v>0</v>
-      </c>
-      <c r="M40" s="3">
+      <c r="L40" s="15">
+        <v>0</v>
+      </c>
+      <c r="M40" s="15">
         <v>0.23100000000000001</v>
       </c>
-      <c r="N40" s="3">
+      <c r="N40" s="15">
         <v>6.7599999999999993E-2</v>
       </c>
-      <c r="O40" s="3">
+      <c r="O40" s="15">
         <v>0.01</v>
       </c>
-      <c r="P40" s="3">
+      <c r="P40" s="15">
         <v>0.36799999999999999</v>
       </c>
     </row>
@@ -9651,43 +9652,43 @@
       <c r="C41" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D41" s="2">
-        <v>0</v>
-      </c>
-      <c r="E41" s="3">
+      <c r="D41" s="15">
+        <v>0</v>
+      </c>
+      <c r="E41" s="15">
         <v>5.8E-4</v>
       </c>
-      <c r="F41" s="3">
+      <c r="F41" s="15">
         <v>3.3999999999999998E-3</v>
       </c>
-      <c r="G41" s="3">
+      <c r="G41" s="15">
         <v>4.2500000000000003E-2</v>
       </c>
-      <c r="H41" s="2">
-        <v>0</v>
-      </c>
-      <c r="I41" s="3">
+      <c r="H41" s="15">
+        <v>0</v>
+      </c>
+      <c r="I41" s="15">
         <v>2E-3</v>
       </c>
-      <c r="J41" s="3">
+      <c r="J41" s="15">
         <v>4.8999999999999998E-3</v>
       </c>
-      <c r="K41" s="3">
+      <c r="K41" s="15">
         <v>0.13100000000000001</v>
       </c>
-      <c r="L41" s="2">
-        <v>0</v>
-      </c>
-      <c r="M41" s="3">
+      <c r="L41" s="15">
+        <v>0</v>
+      </c>
+      <c r="M41" s="15">
         <v>0.35199999999999998</v>
       </c>
-      <c r="N41" s="3">
+      <c r="N41" s="15">
         <v>4.3099999999999999E-2</v>
       </c>
-      <c r="O41" s="3">
+      <c r="O41" s="15">
         <v>4.1999999999999997E-3</v>
       </c>
-      <c r="P41" s="3">
+      <c r="P41" s="15">
         <v>0.28499999999999998</v>
       </c>
     </row>
@@ -9698,43 +9699,43 @@
       <c r="C42" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D42" s="2">
-        <v>0</v>
-      </c>
-      <c r="E42" s="3">
+      <c r="D42" s="15">
+        <v>0</v>
+      </c>
+      <c r="E42" s="15">
         <v>3.8999999999999998E-3</v>
       </c>
-      <c r="F42" s="3">
+      <c r="F42" s="15">
         <v>1.34E-2</v>
       </c>
-      <c r="G42" s="3">
+      <c r="G42" s="15">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="H42" s="2">
-        <v>0</v>
-      </c>
-      <c r="I42" s="3">
+      <c r="H42" s="15">
+        <v>0</v>
+      </c>
+      <c r="I42" s="15">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="J42" s="3">
+      <c r="J42" s="15">
         <v>3.2000000000000002E-3</v>
       </c>
-      <c r="K42" s="3">
+      <c r="K42" s="15">
         <v>0.126</v>
       </c>
-      <c r="L42" s="2">
-        <v>0</v>
-      </c>
-      <c r="M42" s="3">
+      <c r="L42" s="15">
+        <v>0</v>
+      </c>
+      <c r="M42" s="15">
         <v>0.186</v>
       </c>
-      <c r="N42" s="3">
+      <c r="N42" s="15">
         <v>4.3200000000000002E-2</v>
       </c>
-      <c r="O42" s="3">
+      <c r="O42" s="15">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="P42" s="3">
+      <c r="P42" s="15">
         <v>0.47699999999999998</v>
       </c>
     </row>
@@ -9745,43 +9746,43 @@
       <c r="C43" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D43" s="2">
-        <v>0</v>
-      </c>
-      <c r="E43" s="2">
-        <v>0</v>
-      </c>
-      <c r="F43" s="2">
-        <v>0</v>
-      </c>
-      <c r="G43" s="2">
-        <v>0</v>
-      </c>
-      <c r="H43" s="2">
-        <v>0</v>
-      </c>
-      <c r="I43" s="2">
-        <v>0</v>
-      </c>
-      <c r="J43" s="2">
-        <v>0</v>
-      </c>
-      <c r="K43" s="2">
-        <v>0</v>
-      </c>
-      <c r="L43" s="2">
-        <v>0</v>
-      </c>
-      <c r="M43" s="3">
+      <c r="D43" s="15">
+        <v>0</v>
+      </c>
+      <c r="E43" s="15">
+        <v>0</v>
+      </c>
+      <c r="F43" s="15">
+        <v>0</v>
+      </c>
+      <c r="G43" s="15">
+        <v>0</v>
+      </c>
+      <c r="H43" s="15">
+        <v>0</v>
+      </c>
+      <c r="I43" s="15">
+        <v>0</v>
+      </c>
+      <c r="J43" s="15">
+        <v>0</v>
+      </c>
+      <c r="K43" s="15">
+        <v>0</v>
+      </c>
+      <c r="L43" s="15">
+        <v>0</v>
+      </c>
+      <c r="M43" s="15">
         <v>0.995</v>
       </c>
-      <c r="N43" s="2">
-        <v>0</v>
-      </c>
-      <c r="O43" s="2">
-        <v>0</v>
-      </c>
-      <c r="P43" s="2">
+      <c r="N43" s="15">
+        <v>0</v>
+      </c>
+      <c r="O43" s="15">
+        <v>0</v>
+      </c>
+      <c r="P43" s="15">
         <v>0</v>
       </c>
     </row>
@@ -9792,43 +9793,43 @@
       <c r="C44" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D44" s="2">
-        <v>0</v>
-      </c>
-      <c r="E44" s="2">
-        <v>0</v>
-      </c>
-      <c r="F44" s="3">
+      <c r="D44" s="15">
+        <v>0</v>
+      </c>
+      <c r="E44" s="15">
+        <v>0</v>
+      </c>
+      <c r="F44" s="15">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="G44" s="3">
+      <c r="G44" s="15">
         <v>2.2200000000000001E-2</v>
       </c>
-      <c r="H44" s="2">
-        <v>0</v>
-      </c>
-      <c r="I44" s="3">
+      <c r="H44" s="15">
+        <v>0</v>
+      </c>
+      <c r="I44" s="15">
         <v>3.1E-4</v>
       </c>
-      <c r="J44" s="3">
+      <c r="J44" s="15">
         <v>7.6999999999999996E-4</v>
       </c>
-      <c r="K44" s="3">
+      <c r="K44" s="15">
         <v>6.5299999999999997E-2</v>
       </c>
-      <c r="L44" s="2">
-        <v>0</v>
-      </c>
-      <c r="M44" s="3">
+      <c r="L44" s="15">
+        <v>0</v>
+      </c>
+      <c r="M44" s="15">
         <v>0.56999999999999995</v>
       </c>
-      <c r="N44" s="3">
+      <c r="N44" s="15">
         <v>1.46E-2</v>
       </c>
-      <c r="O44" s="2">
-        <v>0</v>
-      </c>
-      <c r="P44" s="3">
+      <c r="O44" s="15">
+        <v>0</v>
+      </c>
+      <c r="P44" s="15">
         <v>0.29399999999999998</v>
       </c>
     </row>
@@ -9839,43 +9840,43 @@
       <c r="C45" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D45" s="2">
-        <v>0</v>
-      </c>
-      <c r="E45" s="2">
-        <v>0</v>
-      </c>
-      <c r="F45" s="3">
+      <c r="D45" s="15">
+        <v>0</v>
+      </c>
+      <c r="E45" s="15">
+        <v>0</v>
+      </c>
+      <c r="F45" s="15">
         <v>1.06E-2</v>
       </c>
-      <c r="G45" s="3">
+      <c r="G45" s="15">
         <v>4.4400000000000002E-2</v>
       </c>
-      <c r="H45" s="2">
-        <v>0</v>
-      </c>
-      <c r="I45" s="3">
+      <c r="H45" s="15">
+        <v>0</v>
+      </c>
+      <c r="I45" s="15">
         <v>6.3000000000000003E-4</v>
       </c>
-      <c r="J45" s="3">
+      <c r="J45" s="15">
         <v>1.2999999999999999E-3</v>
       </c>
-      <c r="K45" s="3">
+      <c r="K45" s="15">
         <v>5.91E-2</v>
       </c>
-      <c r="L45" s="2">
-        <v>0</v>
-      </c>
-      <c r="M45" s="3">
+      <c r="L45" s="15">
+        <v>0</v>
+      </c>
+      <c r="M45" s="15">
         <v>0.39600000000000002</v>
       </c>
-      <c r="N45" s="3">
+      <c r="N45" s="15">
         <v>2.47E-2</v>
       </c>
-      <c r="O45" s="3">
+      <c r="O45" s="15">
         <v>3.1E-4</v>
       </c>
-      <c r="P45" s="3">
+      <c r="P45" s="15">
         <v>0.39900000000000002</v>
       </c>
     </row>
@@ -9886,43 +9887,43 @@
       <c r="C46" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D46" s="2">
-        <v>0</v>
-      </c>
-      <c r="E46" s="3">
+      <c r="D46" s="15">
+        <v>0</v>
+      </c>
+      <c r="E46" s="15">
         <v>5.1999999999999995E-4</v>
       </c>
-      <c r="F46" s="3">
+      <c r="F46" s="15">
         <v>7.6E-3</v>
       </c>
-      <c r="G46" s="3">
+      <c r="G46" s="15">
         <v>3.56E-2</v>
       </c>
-      <c r="H46" s="2">
-        <v>0</v>
-      </c>
-      <c r="I46" s="3">
+      <c r="H46" s="15">
+        <v>0</v>
+      </c>
+      <c r="I46" s="15">
         <v>1.7000000000000001E-4</v>
       </c>
-      <c r="J46" s="3">
+      <c r="J46" s="15">
         <v>9.2000000000000003E-4</v>
       </c>
-      <c r="K46" s="3">
+      <c r="K46" s="15">
         <v>6.6400000000000001E-2</v>
       </c>
-      <c r="L46" s="2">
-        <v>0</v>
-      </c>
-      <c r="M46" s="3">
+      <c r="L46" s="15">
+        <v>0</v>
+      </c>
+      <c r="M46" s="15">
         <v>0.433</v>
       </c>
-      <c r="N46" s="3">
+      <c r="N46" s="15">
         <v>1.34E-2</v>
       </c>
-      <c r="O46" s="4">
+      <c r="O46" s="15">
         <v>5.7800000000000002E-5</v>
       </c>
-      <c r="P46" s="3">
+      <c r="P46" s="15">
         <v>0.42499999999999999</v>
       </c>
     </row>
@@ -9933,43 +9934,43 @@
       <c r="C47" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D47" s="2">
-        <v>0</v>
-      </c>
-      <c r="E47" s="2">
-        <v>0</v>
-      </c>
-      <c r="F47" s="3">
+      <c r="D47" s="15">
+        <v>0</v>
+      </c>
+      <c r="E47" s="15">
+        <v>0</v>
+      </c>
+      <c r="F47" s="15">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="G47" s="3">
+      <c r="G47" s="15">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="H47" s="2">
-        <v>0</v>
-      </c>
-      <c r="I47" s="2">
-        <v>0</v>
-      </c>
-      <c r="J47" s="3">
+      <c r="H47" s="15">
+        <v>0</v>
+      </c>
+      <c r="I47" s="15">
+        <v>0</v>
+      </c>
+      <c r="J47" s="15">
         <v>5.1000000000000004E-4</v>
       </c>
-      <c r="K47" s="3">
+      <c r="K47" s="15">
         <v>5.4100000000000002E-2</v>
       </c>
-      <c r="L47" s="2">
-        <v>0</v>
-      </c>
-      <c r="M47" s="3">
+      <c r="L47" s="15">
+        <v>0</v>
+      </c>
+      <c r="M47" s="15">
         <v>0.77</v>
       </c>
-      <c r="N47" s="3">
+      <c r="N47" s="15">
         <v>1.7899999999999999E-2</v>
       </c>
-      <c r="O47" s="2">
-        <v>0</v>
-      </c>
-      <c r="P47" s="3">
+      <c r="O47" s="15">
+        <v>0</v>
+      </c>
+      <c r="P47" s="15">
         <v>0.127</v>
       </c>
     </row>
@@ -9980,43 +9981,43 @@
       <c r="C48" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D48" s="2">
-        <v>0</v>
-      </c>
-      <c r="E48" s="2">
-        <v>0</v>
-      </c>
-      <c r="F48" s="3">
+      <c r="D48" s="15">
+        <v>0</v>
+      </c>
+      <c r="E48" s="15">
+        <v>0</v>
+      </c>
+      <c r="F48" s="15">
         <v>1.1900000000000001E-2</v>
       </c>
-      <c r="G48" s="3">
+      <c r="G48" s="15">
         <v>2.3400000000000001E-2</v>
       </c>
-      <c r="H48" s="2">
-        <v>0</v>
-      </c>
-      <c r="I48" s="2">
-        <v>0</v>
-      </c>
-      <c r="J48" s="3">
+      <c r="H48" s="15">
+        <v>0</v>
+      </c>
+      <c r="I48" s="15">
+        <v>0</v>
+      </c>
+      <c r="J48" s="15">
         <v>9.8999999999999999E-4</v>
       </c>
-      <c r="K48" s="3">
+      <c r="K48" s="15">
         <v>8.6999999999999994E-2</v>
       </c>
-      <c r="L48" s="2">
-        <v>0</v>
-      </c>
-      <c r="M48" s="3">
+      <c r="L48" s="15">
+        <v>0</v>
+      </c>
+      <c r="M48" s="15">
         <v>0.371</v>
       </c>
-      <c r="N48" s="3">
+      <c r="N48" s="15">
         <v>2.4899999999999999E-2</v>
       </c>
-      <c r="O48" s="3">
+      <c r="O48" s="15">
         <v>2.5000000000000001E-4</v>
       </c>
-      <c r="P48" s="3">
+      <c r="P48" s="15">
         <v>0.45100000000000001</v>
       </c>
     </row>
@@ -10027,43 +10028,43 @@
       <c r="C49" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D49" s="2">
-        <v>0</v>
-      </c>
-      <c r="E49" s="3">
+      <c r="D49" s="15">
+        <v>0</v>
+      </c>
+      <c r="E49" s="15">
         <v>1.2E-4</v>
       </c>
-      <c r="F49" s="3">
+      <c r="F49" s="15">
         <v>5.7999999999999996E-3</v>
       </c>
-      <c r="G49" s="3">
+      <c r="G49" s="15">
         <v>3.0200000000000001E-2</v>
       </c>
-      <c r="H49" s="2">
-        <v>0</v>
-      </c>
-      <c r="I49" s="4">
+      <c r="H49" s="15">
+        <v>0</v>
+      </c>
+      <c r="I49" s="15">
         <v>5.77E-5</v>
       </c>
-      <c r="J49" s="3">
+      <c r="J49" s="15">
         <v>8.7000000000000001E-4</v>
       </c>
-      <c r="K49" s="3">
+      <c r="K49" s="15">
         <v>7.7100000000000002E-2</v>
       </c>
-      <c r="L49" s="2">
-        <v>0</v>
-      </c>
-      <c r="M49" s="3">
+      <c r="L49" s="15">
+        <v>0</v>
+      </c>
+      <c r="M49" s="15">
         <v>0.39500000000000002</v>
       </c>
-      <c r="N49" s="3">
+      <c r="N49" s="15">
         <v>1.4500000000000001E-2</v>
       </c>
-      <c r="O49" s="3">
+      <c r="O49" s="15">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="P49" s="3">
+      <c r="P49" s="15">
         <v>0.45800000000000002</v>
       </c>
     </row>

</xml_diff>